<commit_message>
Data: through 2026-10-02, caught up 9/28, 9/29, 10/1 with outcomes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MaxPain_GEX.xlsx
+++ b/MaxPain_GEX.xlsx
@@ -36,8 +36,8 @@
     <numFmt numFmtId="174" formatCode="\+0.0%;\-0.0%;0.0%"/>
     <numFmt numFmtId="175" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="176" formatCode="yyyy-mm-dd hh:mm"/>
-    <numFmt numFmtId="177" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="178" formatCode="+0.0;-0.0"/>
+    <numFmt numFmtId="177" formatCode="+0.0;-0.0"/>
+    <numFmt numFmtId="178" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -383,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -550,7 +550,8 @@
     <xf numFmtId="175" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -953,12 +954,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Max Pain Calc'!$A$2:$A$137</f>
+              <f>'Max Pain Calc'!$A$2:$A$144</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Max Pain Calc'!$B$2:$B$137</f>
+              <f>'Max Pain Calc'!$B$2:$B$144</f>
             </numRef>
           </val>
         </ser>
@@ -1031,12 +1032,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'GEX Calc'!$A$2:$A$79</f>
+              <f>'GEX Calc'!$A$2:$A$99</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'GEX Calc'!$C$2:$C$79</f>
+              <f>'GEX Calc'!$C$2:$C$99</f>
             </numRef>
           </val>
         </ser>
@@ -1384,7 +1385,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>190</v>
+        <v>79</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
@@ -1393,7 +1394,7 @@
       </c>
       <c r="F2" s="26" t="inlineStr">
         <is>
-          <t>BB1 Week 1 - OCT 2026 (V26)</t>
+          <t>MW1 Week 1 - OCT 2026 (V26)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -1410,7 +1411,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
@@ -1418,7 +1419,7 @@
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
@@ -1442,7 +1443,7 @@
         </is>
       </c>
       <c r="F4" s="26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
@@ -1458,7 +1459,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
@@ -1466,7 +1467,7 @@
         </is>
       </c>
       <c r="F5" s="26" t="n">
-        <v>3048</v>
+        <v>3565</v>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
@@ -1476,7 +1477,7 @@
     </row>
     <row r="6" ht="25.5" customHeight="1" s="61">
       <c r="A6" s="2" t="n">
-        <v>3870</v>
+        <v>3805</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>0</v>
@@ -1490,7 +1491,7 @@
         </is>
       </c>
       <c r="F6" s="26" t="n">
-        <v>3400</v>
+        <v>2801</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
@@ -1500,29 +1501,29 @@
     </row>
     <row r="7" ht="15" customHeight="1" s="61">
       <c r="A7" s="2" t="n">
-        <v>3875</v>
+        <v>3820</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="61">
       <c r="A8" s="2" t="n">
-        <v>3900</v>
+        <v>3825</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="61">
       <c r="A9" s="2" t="n">
-        <v>3905</v>
+        <v>3880</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>0</v>
@@ -1533,95 +1534,95 @@
     </row>
     <row r="10" ht="15" customHeight="1" s="61">
       <c r="A10" s="2" t="n">
-        <v>3920</v>
+        <v>3895</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="61">
       <c r="A11" s="2" t="n">
-        <v>3925</v>
+        <v>3900</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="61">
       <c r="A12" s="2" t="n">
-        <v>3935</v>
+        <v>3905</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="61">
       <c r="A13" s="2" t="n">
-        <v>3940</v>
+        <v>3915</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="61">
       <c r="A14" s="2" t="n">
-        <v>3950</v>
+        <v>3925</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="61">
       <c r="A15" s="2" t="n">
-        <v>3965</v>
+        <v>3935</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="61">
       <c r="A16" s="2" t="n">
-        <v>3970</v>
+        <v>3940</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="61">
       <c r="A17" s="2" t="n">
-        <v>3975</v>
+        <v>3950</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>26</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="61">
       <c r="A18" s="2" t="n">
-        <v>3980</v>
+        <v>3955</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>0</v>
@@ -1632,117 +1633,117 @@
     </row>
     <row r="19" ht="15" customHeight="1" s="61">
       <c r="A19" s="2" t="n">
-        <v>3985</v>
+        <v>3960</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="61">
       <c r="A20" s="2" t="n">
-        <v>3990</v>
+        <v>3965</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="61">
       <c r="A21" s="2" t="n">
-        <v>4000</v>
+        <v>3970</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>58</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="61">
       <c r="A22" s="2" t="n">
-        <v>4010</v>
+        <v>3975</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C22" s="3" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="61">
       <c r="A23" s="2" t="n">
-        <v>4015</v>
+        <v>3980</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="61">
       <c r="A24" s="2" t="n">
-        <v>4020</v>
+        <v>3985</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C24" s="3" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="61">
       <c r="A25" s="2" t="n">
-        <v>4025</v>
+        <v>3995</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>46</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="61">
       <c r="A26" s="2" t="n">
-        <v>4030</v>
+        <v>4000</v>
       </c>
       <c r="B26" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>15</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="61">
       <c r="A27" s="2" t="n">
-        <v>4035</v>
+        <v>4005</v>
       </c>
       <c r="B27" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="61">
       <c r="A28" s="2" t="n">
-        <v>4040</v>
+        <v>4010</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C28" s="3" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="61">
       <c r="A29" s="2" t="n">
-        <v>4045</v>
+        <v>4015</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0</v>
@@ -1753,51 +1754,51 @@
     </row>
     <row r="30" ht="15" customHeight="1" s="61">
       <c r="A30" s="2" t="n">
-        <v>4050</v>
+        <v>4020</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C30" s="3" t="n">
-        <v>72</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="61">
       <c r="A31" s="2" t="n">
-        <v>4055</v>
+        <v>4025</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C31" s="3" t="n">
-        <v>3</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="61">
       <c r="A32" s="2" t="n">
-        <v>4060</v>
+        <v>4030</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="61">
       <c r="A33" s="2" t="n">
-        <v>4065</v>
+        <v>4035</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="61">
       <c r="A34" s="2" t="n">
-        <v>4070</v>
+        <v>4040</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>0</v>
@@ -1808,472 +1809,472 @@
     </row>
     <row r="35" ht="15" customHeight="1" s="61">
       <c r="A35" s="2" t="n">
-        <v>4075</v>
+        <v>4045</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="61">
       <c r="A36" s="2" t="n">
-        <v>4080</v>
+        <v>4050</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>5</v>
+        <v>344</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="61">
       <c r="A37" s="2" t="n">
-        <v>4085</v>
+        <v>4055</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="61">
       <c r="A38" s="2" t="n">
-        <v>4090</v>
+        <v>4060</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>305</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="61">
       <c r="A39" s="2" t="n">
-        <v>4095</v>
+        <v>4065</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>143</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="61">
       <c r="A40" s="2" t="n">
-        <v>4100</v>
+        <v>4070</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C40" s="3" t="n">
-        <v>82</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="61">
       <c r="A41" s="2" t="n">
-        <v>4105</v>
+        <v>4075</v>
       </c>
       <c r="B41" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C41" s="3" t="n">
-        <v>7</v>
+        <v>242</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="61">
       <c r="A42" s="2" t="n">
-        <v>4110</v>
+        <v>4080</v>
       </c>
       <c r="B42" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C42" s="3" t="n">
-        <v>132</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="61">
       <c r="A43" s="2" t="n">
-        <v>4115</v>
+        <v>4085</v>
       </c>
       <c r="B43" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="61">
       <c r="A44" s="2" t="n">
-        <v>4120</v>
+        <v>4090</v>
       </c>
       <c r="B44" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C44" s="3" t="n">
-        <v>83</v>
+        <v>22</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="61">
       <c r="A45" s="2" t="n">
-        <v>4125</v>
+        <v>4095</v>
       </c>
       <c r="B45" s="3" t="n">
         <v>0</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>67</v>
+        <v>5</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="61">
       <c r="A46" s="2" t="n">
-        <v>4130</v>
+        <v>4100</v>
       </c>
       <c r="B46" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>73</v>
+        <v>237</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="61">
       <c r="A47" s="2" t="n">
-        <v>4135</v>
+        <v>4105</v>
       </c>
       <c r="B47" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="61">
       <c r="A48" s="2" t="n">
-        <v>4140</v>
+        <v>4110</v>
       </c>
       <c r="B48" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C48" s="3" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="61">
       <c r="A49" s="2" t="n">
-        <v>4145</v>
+        <v>4115</v>
       </c>
       <c r="B49" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C49" s="3" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="61">
       <c r="A50" s="2" t="n">
-        <v>4150</v>
+        <v>4120</v>
       </c>
       <c r="B50" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C50" s="3" t="n">
-        <v>112</v>
+        <v>19</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="61">
       <c r="A51" s="2" t="n">
-        <v>4155</v>
+        <v>4125</v>
       </c>
       <c r="B51" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C51" s="3" t="n">
-        <v>37</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="61">
       <c r="A52" s="2" t="n">
-        <v>4160</v>
+        <v>4130</v>
       </c>
       <c r="B52" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C52" s="3" t="n">
-        <v>42</v>
+        <v>18</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>4165</v>
+        <v>4135</v>
       </c>
       <c r="B53" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C53" s="3" t="n">
-        <v>46</v>
+        <v>11</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="61">
       <c r="A54" s="2" t="n">
-        <v>4170</v>
+        <v>4140</v>
       </c>
       <c r="B54" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C54" s="3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="61">
       <c r="A55" s="2" t="n">
-        <v>4175</v>
+        <v>4145</v>
       </c>
       <c r="B55" s="3" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="C55" s="3" t="n">
-        <v>108</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="61">
       <c r="A56" s="2" t="n">
-        <v>4180</v>
+        <v>4150</v>
       </c>
       <c r="B56" s="3" t="n">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="C56" s="3" t="n">
-        <v>45</v>
+        <v>153</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>4185</v>
+        <v>4155</v>
       </c>
       <c r="B57" s="3" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="C57" s="3" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>4190</v>
+        <v>4160</v>
       </c>
       <c r="B58" s="3" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C58" s="3" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>4195</v>
+        <v>4165</v>
       </c>
       <c r="B59" s="3" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C59" s="3" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>4200</v>
+        <v>4170</v>
       </c>
       <c r="B60" s="3" t="n">
-        <v>208</v>
+        <v>56</v>
       </c>
       <c r="C60" s="3" t="n">
-        <v>247</v>
+        <v>103</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>4205</v>
+        <v>4175</v>
       </c>
       <c r="B61" s="3" t="n">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="C61" s="3" t="n">
-        <v>12</v>
+        <v>95</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>4210</v>
+        <v>4180</v>
       </c>
       <c r="B62" s="3" t="n">
-        <v>77</v>
+        <v>9</v>
       </c>
       <c r="C62" s="3" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>4215</v>
+        <v>4185</v>
       </c>
       <c r="B63" t="n">
-        <v>53</v>
+        <v>9</v>
       </c>
       <c r="C63" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>4220</v>
+        <v>4190</v>
       </c>
       <c r="B64" t="n">
-        <v>53</v>
+        <v>111</v>
       </c>
       <c r="C64" t="n">
-        <v>45</v>
+        <v>17</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>4225</v>
+        <v>4195</v>
       </c>
       <c r="B65" t="n">
-        <v>111</v>
+        <v>46</v>
       </c>
       <c r="C65" t="n">
-        <v>295</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>4230</v>
+        <v>4200</v>
       </c>
       <c r="B66" t="n">
-        <v>136</v>
+        <v>82</v>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>4235</v>
+        <v>4205</v>
       </c>
       <c r="B67" t="n">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="C67" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>4240</v>
+        <v>4210</v>
       </c>
       <c r="B68" t="n">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>4245</v>
+        <v>4215</v>
       </c>
       <c r="B69" t="n">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="C69" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>4250</v>
+        <v>4220</v>
       </c>
       <c r="B70" t="n">
-        <v>116</v>
+        <v>169</v>
       </c>
       <c r="C70" t="n">
-        <v>202</v>
+        <v>23</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>4255</v>
+        <v>4225</v>
       </c>
       <c r="B71" t="n">
-        <v>54</v>
+        <v>161</v>
       </c>
       <c r="C71" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>4260</v>
+        <v>4230</v>
       </c>
       <c r="B72" t="n">
         <v>52</v>
       </c>
       <c r="C72" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>4265</v>
+        <v>4235</v>
       </c>
       <c r="B73" t="n">
-        <v>2</v>
+        <v>126</v>
       </c>
       <c r="C73" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>4270</v>
+        <v>4240</v>
       </c>
       <c r="B74" t="n">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>4275</v>
+        <v>4245</v>
       </c>
       <c r="B75" t="n">
-        <v>26</v>
+        <v>8</v>
       </c>
       <c r="C75" t="n">
-        <v>98</v>
+        <v>1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>4280</v>
+        <v>4250</v>
       </c>
       <c r="B76" t="n">
-        <v>38</v>
+        <v>104</v>
       </c>
       <c r="C76" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>4285</v>
+        <v>4255</v>
       </c>
       <c r="B77" t="n">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C77" t="n">
         <v>0</v>
@@ -2281,54 +2282,54 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>4290</v>
+        <v>4260</v>
       </c>
       <c r="B78" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>4295</v>
+        <v>4265</v>
       </c>
       <c r="B79" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="C79" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>4300</v>
+        <v>4270</v>
       </c>
       <c r="B80" t="n">
-        <v>118</v>
+        <v>21</v>
       </c>
       <c r="C80" t="n">
-        <v>112</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>4305</v>
+        <v>4275</v>
       </c>
       <c r="B81" t="n">
-        <v>13</v>
+        <v>84</v>
       </c>
       <c r="C81" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>4310</v>
+        <v>4280</v>
       </c>
       <c r="B82" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="C82" t="n">
         <v>1</v>
@@ -2336,10 +2337,10 @@
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>4315</v>
+        <v>4285</v>
       </c>
       <c r="B83" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C83" t="n">
         <v>0</v>
@@ -2347,10 +2348,10 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>4320</v>
+        <v>4290</v>
       </c>
       <c r="B84" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C84" t="n">
         <v>0</v>
@@ -2358,54 +2359,54 @@
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>4325</v>
+        <v>4295</v>
       </c>
       <c r="B85" t="n">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="C85" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>4330</v>
+        <v>4300</v>
       </c>
       <c r="B86" t="n">
-        <v>15</v>
+        <v>164</v>
       </c>
       <c r="C86" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>4335</v>
+        <v>4305</v>
       </c>
       <c r="B87" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>4340</v>
+        <v>4310</v>
       </c>
       <c r="B88" t="n">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="C88" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>4345</v>
+        <v>4315</v>
       </c>
       <c r="B89" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C89" t="n">
         <v>0</v>
@@ -2413,76 +2414,76 @@
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>4350</v>
+        <v>4320</v>
       </c>
       <c r="B90" t="n">
-        <v>94</v>
+        <v>12</v>
       </c>
       <c r="C90" t="n">
-        <v>52</v>
+        <v>2</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>4360</v>
+        <v>4325</v>
       </c>
       <c r="B91" t="n">
-        <v>3</v>
+        <v>82</v>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>69</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>4370</v>
+        <v>4330</v>
       </c>
       <c r="B92" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C92" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>4375</v>
+        <v>4335</v>
       </c>
       <c r="B93" t="n">
-        <v>289</v>
+        <v>2</v>
       </c>
       <c r="C93" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>4380</v>
+        <v>4340</v>
       </c>
       <c r="B94" t="n">
+        <v>2</v>
+      </c>
+      <c r="C94" t="n">
         <v>1</v>
-      </c>
-      <c r="C94" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>4385</v>
+        <v>4350</v>
       </c>
       <c r="B95" t="n">
-        <v>26</v>
+        <v>373</v>
       </c>
       <c r="C95" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>4390</v>
+        <v>4355</v>
       </c>
       <c r="B96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C96" t="n">
         <v>0</v>
@@ -2490,10 +2491,10 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>4395</v>
+        <v>4360</v>
       </c>
       <c r="B97" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C97" t="n">
         <v>0</v>
@@ -2501,21 +2502,21 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>4400</v>
+        <v>4365</v>
       </c>
       <c r="B98" t="n">
-        <v>119</v>
+        <v>2</v>
       </c>
       <c r="C98" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>4405</v>
+        <v>4370</v>
       </c>
       <c r="B99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C99" t="n">
         <v>0</v>
@@ -2523,21 +2524,21 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>4410</v>
+        <v>4375</v>
       </c>
       <c r="B100" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C100" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>4420</v>
+        <v>4380</v>
       </c>
       <c r="B101" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C101" t="n">
         <v>0</v>
@@ -2545,43 +2546,43 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>4425</v>
+        <v>4390</v>
       </c>
       <c r="B102" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="C102" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>4435</v>
+        <v>4400</v>
       </c>
       <c r="B103" t="n">
-        <v>5</v>
+        <v>378</v>
       </c>
       <c r="C103" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>4450</v>
+        <v>4415</v>
       </c>
       <c r="B104" t="n">
-        <v>158</v>
+        <v>16</v>
       </c>
       <c r="C104" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>4455</v>
+        <v>4420</v>
       </c>
       <c r="B105" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C105" t="n">
         <v>0</v>
@@ -2589,43 +2590,43 @@
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>4460</v>
+        <v>4425</v>
       </c>
       <c r="B106" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C106" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>4475</v>
+        <v>4430</v>
       </c>
       <c r="B107" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="C107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>4500</v>
+        <v>4435</v>
       </c>
       <c r="B108" t="n">
-        <v>137</v>
+        <v>5</v>
       </c>
       <c r="C108" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>4505</v>
+        <v>4440</v>
       </c>
       <c r="B109" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C109" t="n">
         <v>0</v>
@@ -2633,10 +2634,10 @@
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>4525</v>
+        <v>4445</v>
       </c>
       <c r="B110" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C110" t="n">
         <v>0</v>
@@ -2644,21 +2645,21 @@
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>4550</v>
+        <v>4450</v>
       </c>
       <c r="B111" t="n">
-        <v>22</v>
+        <v>100</v>
       </c>
       <c r="C111" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>4560</v>
+        <v>4455</v>
       </c>
       <c r="B112" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C112" t="n">
         <v>0</v>
@@ -2666,10 +2667,10 @@
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>4575</v>
+        <v>4460</v>
       </c>
       <c r="B113" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="C113" t="n">
         <v>0</v>
@@ -2677,10 +2678,10 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>4600</v>
+        <v>4475</v>
       </c>
       <c r="B114" t="n">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="C114" t="n">
         <v>0</v>
@@ -2688,10 +2689,10 @@
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>4625</v>
+        <v>4480</v>
       </c>
       <c r="B115" t="n">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="C115" t="n">
         <v>0</v>
@@ -2699,10 +2700,10 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>4650</v>
+        <v>4485</v>
       </c>
       <c r="B116" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C116" t="n">
         <v>0</v>
@@ -2710,21 +2711,21 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>4675</v>
+        <v>4500</v>
       </c>
       <c r="B117" t="n">
-        <v>14</v>
+        <v>237</v>
       </c>
       <c r="C117" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>4700</v>
+        <v>4520</v>
       </c>
       <c r="B118" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="C118" t="n">
         <v>0</v>
@@ -2732,32 +2733,32 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>4725</v>
+        <v>4525</v>
       </c>
       <c r="B119" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C119" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>4750</v>
+        <v>4550</v>
       </c>
       <c r="B120" t="n">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="C120" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>4775</v>
+        <v>4575</v>
       </c>
       <c r="B121" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C121" t="n">
         <v>0</v>
@@ -2765,21 +2766,21 @@
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>4800</v>
+        <v>4600</v>
       </c>
       <c r="B122" t="n">
-        <v>18</v>
+        <v>93</v>
       </c>
       <c r="C122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>4825</v>
+        <v>4625</v>
       </c>
       <c r="B123" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="C123" t="n">
         <v>0</v>
@@ -2787,10 +2788,10 @@
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>4850</v>
+        <v>4650</v>
       </c>
       <c r="B124" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C124" t="n">
         <v>0</v>
@@ -2798,10 +2799,10 @@
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>4900</v>
+        <v>4675</v>
       </c>
       <c r="B125" t="n">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="C125" t="n">
         <v>0</v>
@@ -2809,10 +2810,10 @@
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>4925</v>
+        <v>4700</v>
       </c>
       <c r="B126" t="n">
-        <v>3</v>
+        <v>57</v>
       </c>
       <c r="C126" t="n">
         <v>0</v>
@@ -2820,10 +2821,10 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>4950</v>
+        <v>4725</v>
       </c>
       <c r="B127" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C127" t="n">
         <v>0</v>
@@ -2831,10 +2832,10 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>4975</v>
+        <v>4750</v>
       </c>
       <c r="B128" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C128" t="n">
         <v>0</v>
@@ -2842,21 +2843,21 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>5000</v>
+        <v>4775</v>
       </c>
       <c r="B129" t="n">
-        <v>3</v>
+        <v>52</v>
       </c>
       <c r="C129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>5025</v>
+        <v>4800</v>
       </c>
       <c r="B130" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C130" t="n">
         <v>0</v>
@@ -2864,10 +2865,10 @@
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>5050</v>
+        <v>4825</v>
       </c>
       <c r="B131" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C131" t="n">
         <v>0</v>
@@ -2875,10 +2876,10 @@
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>5100</v>
+        <v>4850</v>
       </c>
       <c r="B132" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C132" t="n">
         <v>0</v>
@@ -2886,10 +2887,10 @@
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>5125</v>
+        <v>4900</v>
       </c>
       <c r="B133" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C133" t="n">
         <v>0</v>
@@ -2897,10 +2898,10 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>5200</v>
+        <v>4925</v>
       </c>
       <c r="B134" t="n">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="C134" t="n">
         <v>0</v>
@@ -2908,10 +2909,10 @@
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>5250</v>
+        <v>4950</v>
       </c>
       <c r="B135" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C135" t="n">
         <v>0</v>
@@ -2919,10 +2920,10 @@
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>5300</v>
+        <v>4975</v>
       </c>
       <c r="B136" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C136" t="n">
         <v>0</v>
@@ -2930,22 +2931,92 @@
     </row>
     <row r="137">
       <c r="A137" t="n">
+        <v>5000</v>
+      </c>
+      <c r="B137" t="n">
+        <v>12</v>
+      </c>
+      <c r="C137" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>5100</v>
+      </c>
+      <c r="B138" t="n">
+        <v>13</v>
+      </c>
+      <c r="C138" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>5200</v>
+      </c>
+      <c r="B139" t="n">
+        <v>2</v>
+      </c>
+      <c r="C139" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>5250</v>
+      </c>
+      <c r="B140" t="n">
+        <v>7</v>
+      </c>
+      <c r="C140" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>5300</v>
+      </c>
+      <c r="B141" t="n">
+        <v>11</v>
+      </c>
+      <c r="C141" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
         <v>5400</v>
       </c>
-      <c r="B137" t="n">
-        <v>3</v>
-      </c>
-      <c r="C137" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
+      <c r="B142" t="n">
+        <v>11</v>
+      </c>
+      <c r="C142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>5500</v>
+      </c>
+      <c r="B143" t="n">
+        <v>8</v>
+      </c>
+      <c r="C143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>5750</v>
+      </c>
+      <c r="B144" t="n">
+        <v>40</v>
+      </c>
+      <c r="C144" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="145"/>
     <row r="146"/>
     <row r="147"/>
@@ -3127,7 +3198,7 @@
         </is>
       </c>
       <c r="F4" s="13" t="n">
-        <v>4186.7</v>
+        <v>4162.3</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="61">
@@ -6223,7 +6294,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.42578125" bestFit="1" customWidth="1" style="61" min="1" max="1"/>
@@ -6455,43 +6526,219 @@
     </row>
     <row r="6">
       <c r="A6" s="71" t="n">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BB1 Week 1 - OCT 2026 (V26)</t>
+          <t>AB1 Week 5 - SEP 2026 (U26)</t>
         </is>
       </c>
       <c r="C6" s="29" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="30" t="n">
-        <v>4186.7</v>
+        <v>4136.4</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>4230</v>
+        <v>4200</v>
       </c>
       <c r="F6" s="31" t="n">
-        <v>0.01034227434494953</v>
+        <v>0.01537568900493191</v>
       </c>
       <c r="G6" s="29" t="n">
         <v>4</v>
       </c>
       <c r="H6" s="32" t="n">
-        <v>1.115485564304462</v>
+        <v>0.8211080160940886</v>
       </c>
       <c r="I6" s="33" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
+          <t>FINAL</t>
+        </is>
+      </c>
+      <c r="K6" s="73" t="n">
+        <v>46298.65218100695</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>OCT 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="71" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>WD1 Week 5 - SEP 2026 (U26)</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>4147.7</v>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>4235</v>
+      </c>
+      <c r="F7" s="31" t="n">
+        <v>0.02104780962943322</v>
+      </c>
+      <c r="G7" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" s="32" t="n">
+        <v>0.8326506729081334</v>
+      </c>
+      <c r="I7" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>FINAL</t>
+        </is>
+      </c>
+      <c r="K7" s="73" t="n">
+        <v>46298.65205094907</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>OCT 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="71" t="n">
+        <v>46295</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BB1 Week 1 - OCT 2026 (V26)</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="30" t="n">
+        <v>4186.7</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>4230</v>
+      </c>
+      <c r="F8" s="31" t="n">
+        <v>0.01034227434494953</v>
+      </c>
+      <c r="G8" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="32" t="n">
+        <v>1.115485564304462</v>
+      </c>
+      <c r="I8" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>PRELIMINARY</t>
         </is>
       </c>
-      <c r="K6" s="73" t="n">
+      <c r="K8" s="73" t="n">
         <v>46296.85222474537</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>DEC 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="71" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>E21 Week 1 - OCT 2026 (V26)</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="30" t="n">
+        <v>4202.3</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>4250</v>
+      </c>
+      <c r="F9" s="31" t="n">
+        <v>0.01135092687337882</v>
+      </c>
+      <c r="G9" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="H9" s="32" t="n">
+        <v>1.04210042865891</v>
+      </c>
+      <c r="I9" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>FINAL</t>
+        </is>
+      </c>
+      <c r="K9" s="73" t="n">
+        <v>46298.6519262037</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>DEC 26</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="71" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MW1 Week 1 - OCT 2026 (V26)</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" s="30" t="n">
+        <v>4162.3</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>4215</v>
+      </c>
+      <c r="F10" s="31" t="n">
+        <v>0.01266126900992235</v>
+      </c>
+      <c r="G10" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="32" t="n">
+        <v>0.7856942496493688</v>
+      </c>
+      <c r="I10" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>PRELIMINARY</t>
+        </is>
+      </c>
+      <c r="K10" s="73" t="n">
+        <v>46298.64827216436</v>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>DEC 26</t>
         </is>
@@ -6534,7 +6781,7 @@
     </row>
     <row r="2" ht="15" customHeight="1" s="61">
       <c r="A2" s="36" t="n">
-        <v>4070</v>
+        <v>4020</v>
       </c>
       <c r="B2" s="36" t="n">
         <v>0</v>
@@ -6545,7 +6792,7 @@
     </row>
     <row r="3" ht="15" customHeight="1" s="61">
       <c r="A3" s="36" t="n">
-        <v>4075</v>
+        <v>4025</v>
       </c>
       <c r="B3" s="36" t="n">
         <v>0</v>
@@ -6556,7 +6803,7 @@
     </row>
     <row r="4" ht="15" customHeight="1" s="61">
       <c r="A4" s="36" t="n">
-        <v>4080</v>
+        <v>4030</v>
       </c>
       <c r="B4" s="36" t="n">
         <v>0</v>
@@ -6567,7 +6814,7 @@
     </row>
     <row r="5" ht="15" customHeight="1" s="61">
       <c r="A5" s="36" t="n">
-        <v>4085</v>
+        <v>4035</v>
       </c>
       <c r="B5" s="36" t="n">
         <v>0</v>
@@ -6578,109 +6825,109 @@
     </row>
     <row r="6" ht="15" customHeight="1" s="61">
       <c r="A6" s="36" t="n">
-        <v>4090</v>
+        <v>4040</v>
       </c>
       <c r="B6" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C6" s="36" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="61">
       <c r="A7" s="36" t="n">
-        <v>4095</v>
+        <v>4045</v>
       </c>
       <c r="B7" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="36" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="61">
       <c r="A8" s="36" t="n">
-        <v>4100</v>
+        <v>4050</v>
       </c>
       <c r="B8" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C8" s="36" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="61">
       <c r="A9" s="36" t="n">
-        <v>4105</v>
+        <v>4055</v>
       </c>
       <c r="B9" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C9" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="61">
       <c r="A10" s="36" t="n">
-        <v>4110</v>
+        <v>4060</v>
       </c>
       <c r="B10" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="36" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="61">
       <c r="A11" s="36" t="n">
-        <v>4115</v>
+        <v>4065</v>
       </c>
       <c r="B11" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="61">
       <c r="A12" s="36" t="n">
-        <v>4120</v>
+        <v>4070</v>
       </c>
       <c r="B12" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C12" s="36" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="61">
       <c r="A13" s="36" t="n">
-        <v>4125</v>
+        <v>4075</v>
       </c>
       <c r="B13" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="36" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="61">
       <c r="A14" s="36" t="n">
-        <v>4130</v>
+        <v>4080</v>
       </c>
       <c r="B14" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C14" s="36" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="61">
       <c r="A15" s="36" t="n">
-        <v>4135</v>
+        <v>4085</v>
       </c>
       <c r="B15" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C15" s="36" t="n">
         <v>3</v>
@@ -6688,131 +6935,131 @@
     </row>
     <row r="16" ht="15" customHeight="1" s="61">
       <c r="A16" s="36" t="n">
-        <v>4140</v>
+        <v>4090</v>
       </c>
       <c r="B16" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C16" s="36" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="61">
       <c r="A17" s="36" t="n">
-        <v>4145</v>
+        <v>4095</v>
       </c>
       <c r="B17" s="36" t="n">
         <v>0</v>
       </c>
       <c r="C17" s="36" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="61">
       <c r="A18" s="36" t="n">
-        <v>4150</v>
+        <v>4100</v>
       </c>
       <c r="B18" s="36" t="n">
         <v>1</v>
       </c>
       <c r="C18" s="36" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="61">
       <c r="A19" s="36" t="n">
-        <v>4155</v>
+        <v>4105</v>
       </c>
       <c r="B19" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19" s="36" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="61">
       <c r="A20" s="36" t="n">
-        <v>4160</v>
+        <v>4110</v>
       </c>
       <c r="B20" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="36" t="n">
         <v>1</v>
-      </c>
-      <c r="C20" s="36" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="61">
       <c r="A21" s="36" t="n">
-        <v>4165</v>
+        <v>4115</v>
       </c>
       <c r="B21" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" s="36" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="61">
       <c r="A22" s="36" t="n">
-        <v>4170</v>
+        <v>4120</v>
       </c>
       <c r="B22" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" s="36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="61">
       <c r="A23" s="36" t="n">
-        <v>4175</v>
+        <v>4125</v>
       </c>
       <c r="B23" s="36" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C23" s="36" t="n">
-        <v>37</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="61">
       <c r="A24" s="36" t="n">
-        <v>4180</v>
+        <v>4130</v>
       </c>
       <c r="B24" s="36" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C24" s="36" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="61">
       <c r="A25" s="36" t="n">
-        <v>4185</v>
+        <v>4135</v>
       </c>
       <c r="B25" s="36" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C25" s="36" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="61">
       <c r="A26" s="36" t="n">
-        <v>4190</v>
+        <v>4140</v>
       </c>
       <c r="B26" s="36" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C26" s="36" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="61">
       <c r="A27" s="36" t="n">
-        <v>4195</v>
+        <v>4145</v>
       </c>
       <c r="B27" s="36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="36" t="n">
         <v>2</v>
@@ -6820,131 +7067,131 @@
     </row>
     <row r="28" ht="15" customHeight="1" s="61">
       <c r="A28" s="36" t="n">
-        <v>4200</v>
+        <v>4150</v>
       </c>
       <c r="B28" s="36" t="n">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="C28" s="36" t="n">
-        <v>85</v>
+        <v>46</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="61">
       <c r="A29" s="36" t="n">
-        <v>4205</v>
+        <v>4155</v>
       </c>
       <c r="B29" s="36" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C29" s="36" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="61">
       <c r="A30" s="36" t="n">
-        <v>4210</v>
+        <v>4160</v>
       </c>
       <c r="B30" s="36" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="C30" s="36" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="61">
       <c r="A31" s="36" t="n">
-        <v>4215</v>
+        <v>4165</v>
       </c>
       <c r="B31" s="36" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="C31" s="36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="61">
       <c r="A32" s="36" t="n">
-        <v>4220</v>
+        <v>4170</v>
       </c>
       <c r="B32" s="36" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C32" s="36" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="61">
       <c r="A33" s="36" t="n">
-        <v>4225</v>
+        <v>4175</v>
       </c>
       <c r="B33" s="36" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C33" s="36" t="n">
-        <v>76</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="61">
       <c r="A34" s="36" t="n">
-        <v>4230</v>
+        <v>4180</v>
       </c>
       <c r="B34" s="36" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="C34" s="36" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="61">
       <c r="A35" s="36" t="n">
-        <v>4235</v>
+        <v>4185</v>
       </c>
       <c r="B35" s="36" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C35" s="36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="61">
       <c r="A36" s="36" t="n">
-        <v>4240</v>
+        <v>4190</v>
       </c>
       <c r="B36" s="36" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="C36" s="36" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="61">
       <c r="A37" s="36" t="n">
-        <v>4245</v>
+        <v>4195</v>
       </c>
       <c r="B37" s="36" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C37" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="61">
       <c r="A38" s="36" t="n">
-        <v>4250</v>
+        <v>4200</v>
       </c>
       <c r="B38" s="36" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C38" s="36" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="61">
       <c r="A39" s="36" t="n">
-        <v>4255</v>
+        <v>4205</v>
       </c>
       <c r="B39" s="36" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C39" s="36" t="n">
         <v>0</v>
@@ -6952,87 +7199,87 @@
     </row>
     <row r="40" ht="15" customHeight="1" s="61">
       <c r="A40" s="36" t="n">
-        <v>4260</v>
+        <v>4210</v>
       </c>
       <c r="B40" s="36" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="C40" s="36" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="61">
       <c r="A41" s="36" t="n">
-        <v>4265</v>
+        <v>4215</v>
       </c>
       <c r="B41" s="36" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C41" s="36" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="61">
       <c r="A42" s="36" t="n">
-        <v>4270</v>
+        <v>4220</v>
       </c>
       <c r="B42" s="36" t="n">
+        <v>29</v>
+      </c>
+      <c r="C42" s="36" t="n">
         <v>4</v>
-      </c>
-      <c r="C42" s="36" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="61">
       <c r="A43" s="36" t="n">
-        <v>4275</v>
+        <v>4225</v>
       </c>
       <c r="B43" s="36" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="C43" s="36" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="61">
       <c r="A44" s="36" t="n">
-        <v>4280</v>
+        <v>4230</v>
       </c>
       <c r="B44" s="36" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C44" s="36" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="61">
       <c r="A45" s="36" t="n">
-        <v>4285</v>
+        <v>4235</v>
       </c>
       <c r="B45" s="36" t="n">
+        <v>16</v>
+      </c>
+      <c r="C45" s="36" t="n">
         <v>3</v>
-      </c>
-      <c r="C45" s="36" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="61">
       <c r="A46" s="36" t="n">
-        <v>4290</v>
+        <v>4240</v>
       </c>
       <c r="B46" s="36" t="n">
+        <v>7</v>
+      </c>
+      <c r="C46" s="36" t="n">
         <v>1</v>
-      </c>
-      <c r="C46" s="36" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="61">
       <c r="A47" s="36" t="n">
-        <v>4295</v>
+        <v>4245</v>
       </c>
       <c r="B47" s="36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C47" s="36" t="n">
         <v>0</v>
@@ -7040,21 +7287,21 @@
     </row>
     <row r="48" ht="15" customHeight="1" s="61">
       <c r="A48" s="36" t="n">
-        <v>4300</v>
+        <v>4250</v>
       </c>
       <c r="B48" s="36" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C48" s="36" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="61">
       <c r="A49" s="36" t="n">
-        <v>4305</v>
+        <v>4255</v>
       </c>
       <c r="B49" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C49" s="36" t="n">
         <v>0</v>
@@ -7062,18 +7309,18 @@
     </row>
     <row r="50" ht="15" customHeight="1" s="61">
       <c r="A50" s="36" t="n">
-        <v>4310</v>
+        <v>4260</v>
       </c>
       <c r="B50" s="36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C50" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="61">
       <c r="A51" s="36" t="n">
-        <v>4315</v>
+        <v>4265</v>
       </c>
       <c r="B51" s="36" t="n">
         <v>0</v>
@@ -7084,10 +7331,10 @@
     </row>
     <row r="52" ht="15" customHeight="1" s="61">
       <c r="A52" s="36" t="n">
-        <v>4320</v>
+        <v>4270</v>
       </c>
       <c r="B52" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C52" s="36" t="n">
         <v>0</v>
@@ -7095,21 +7342,21 @@
     </row>
     <row r="53" ht="15" customHeight="1" s="61">
       <c r="A53" s="36" t="n">
-        <v>4325</v>
+        <v>4275</v>
       </c>
       <c r="B53" s="36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C53" s="36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="61">
       <c r="A54" s="36" t="n">
-        <v>4330</v>
+        <v>4280</v>
       </c>
       <c r="B54" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C54" s="36" t="n">
         <v>0</v>
@@ -7117,7 +7364,7 @@
     </row>
     <row r="55" ht="15" customHeight="1" s="61">
       <c r="A55" s="36" t="n">
-        <v>4335</v>
+        <v>4285</v>
       </c>
       <c r="B55" s="36" t="n">
         <v>0</v>
@@ -7128,7 +7375,7 @@
     </row>
     <row r="56" ht="15" customHeight="1" s="61">
       <c r="A56" s="36" t="n">
-        <v>4340</v>
+        <v>4290</v>
       </c>
       <c r="B56" s="36" t="n">
         <v>0</v>
@@ -7139,10 +7386,10 @@
     </row>
     <row r="57" ht="15" customHeight="1" s="61">
       <c r="A57" s="36" t="n">
-        <v>4345</v>
+        <v>4295</v>
       </c>
       <c r="B57" s="36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C57" s="36" t="n">
         <v>0</v>
@@ -7150,21 +7397,21 @@
     </row>
     <row r="58" ht="15" customHeight="1" s="61">
       <c r="A58" s="36" t="n">
-        <v>4350</v>
+        <v>4300</v>
       </c>
       <c r="B58" s="36" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C58" s="36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="61">
       <c r="A59" s="36" t="n">
-        <v>4355</v>
+        <v>4305</v>
       </c>
       <c r="B59" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C59" s="36" t="n">
         <v>0</v>
@@ -7172,10 +7419,10 @@
     </row>
     <row r="60" ht="15" customHeight="1" s="61">
       <c r="A60" s="36" t="n">
-        <v>4360</v>
+        <v>4310</v>
       </c>
       <c r="B60" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C60" s="36" t="n">
         <v>0</v>
@@ -7183,7 +7430,7 @@
     </row>
     <row r="61" ht="15" customHeight="1" s="61">
       <c r="A61" s="36" t="n">
-        <v>4365</v>
+        <v>4315</v>
       </c>
       <c r="B61" s="36" t="n">
         <v>0</v>
@@ -7194,7 +7441,7 @@
     </row>
     <row r="62" ht="15" customHeight="1" s="61">
       <c r="A62" s="36" t="n">
-        <v>4370</v>
+        <v>4320</v>
       </c>
       <c r="B62" s="36" t="n">
         <v>0</v>
@@ -7205,7 +7452,7 @@
     </row>
     <row r="63" ht="15" customHeight="1" s="61">
       <c r="A63" s="36" t="n">
-        <v>4375</v>
+        <v>4325</v>
       </c>
       <c r="B63" s="36" t="n">
         <v>2</v>
@@ -7216,7 +7463,7 @@
     </row>
     <row r="64" ht="15" customHeight="1" s="61">
       <c r="A64" s="36" t="n">
-        <v>4380</v>
+        <v>4330</v>
       </c>
       <c r="B64" s="36" t="n">
         <v>0</v>
@@ -7227,7 +7474,7 @@
     </row>
     <row r="65" ht="15" customHeight="1" s="61">
       <c r="A65" s="36" t="n">
-        <v>4385</v>
+        <v>4335</v>
       </c>
       <c r="B65" s="36" t="n">
         <v>0</v>
@@ -7238,7 +7485,7 @@
     </row>
     <row r="66" ht="15" customHeight="1" s="61">
       <c r="A66" s="36" t="n">
-        <v>4390</v>
+        <v>4340</v>
       </c>
       <c r="B66" s="36" t="n">
         <v>0</v>
@@ -7249,7 +7496,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>4395</v>
+        <v>4345</v>
       </c>
       <c r="B67" t="n">
         <v>0</v>
@@ -7260,18 +7507,18 @@
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>4400</v>
+        <v>4350</v>
       </c>
       <c r="B68" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>4405</v>
+        <v>4355</v>
       </c>
       <c r="B69" t="n">
         <v>0</v>
@@ -7282,7 +7529,7 @@
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>4410</v>
+        <v>4360</v>
       </c>
       <c r="B70" t="n">
         <v>0</v>
@@ -7293,7 +7540,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>4415</v>
+        <v>4365</v>
       </c>
       <c r="B71" t="n">
         <v>0</v>
@@ -7304,7 +7551,7 @@
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>4420</v>
+        <v>4370</v>
       </c>
       <c r="B72" t="n">
         <v>0</v>
@@ -7315,7 +7562,7 @@
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>4425</v>
+        <v>4375</v>
       </c>
       <c r="B73" t="n">
         <v>0</v>
@@ -7326,7 +7573,7 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>4430</v>
+        <v>4380</v>
       </c>
       <c r="B74" t="n">
         <v>0</v>
@@ -7337,7 +7584,7 @@
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>4435</v>
+        <v>4385</v>
       </c>
       <c r="B75" t="n">
         <v>0</v>
@@ -7348,7 +7595,7 @@
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>4440</v>
+        <v>4390</v>
       </c>
       <c r="B76" t="n">
         <v>0</v>
@@ -7359,7 +7606,7 @@
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>4445</v>
+        <v>4395</v>
       </c>
       <c r="B77" t="n">
         <v>0</v>
@@ -7370,10 +7617,10 @@
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>4450</v>
+        <v>4400</v>
       </c>
       <c r="B78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C78" t="n">
         <v>0</v>
@@ -7381,35 +7628,235 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
+        <v>4405</v>
+      </c>
+      <c r="B79" t="n">
+        <v>0</v>
+      </c>
+      <c r="C79" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>4410</v>
+      </c>
+      <c r="B80" t="n">
+        <v>0</v>
+      </c>
+      <c r="C80" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>4415</v>
+      </c>
+      <c r="B81" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>4420</v>
+      </c>
+      <c r="B82" t="n">
+        <v>0</v>
+      </c>
+      <c r="C82" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>4425</v>
+      </c>
+      <c r="B83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>4430</v>
+      </c>
+      <c r="B84" t="n">
+        <v>0</v>
+      </c>
+      <c r="C84" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>4435</v>
+      </c>
+      <c r="B85" t="n">
+        <v>0</v>
+      </c>
+      <c r="C85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>4440</v>
+      </c>
+      <c r="B86" t="n">
+        <v>0</v>
+      </c>
+      <c r="C86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>4445</v>
+      </c>
+      <c r="B87" t="n">
+        <v>0</v>
+      </c>
+      <c r="C87" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>4450</v>
+      </c>
+      <c r="B88" t="n">
+        <v>0</v>
+      </c>
+      <c r="C88" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
         <v>4455</v>
       </c>
-      <c r="B79" t="n">
-        <v>0</v>
-      </c>
-      <c r="C79" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
+      <c r="B89" t="n">
+        <v>0</v>
+      </c>
+      <c r="C89" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>4460</v>
+      </c>
+      <c r="B90" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>4465</v>
+      </c>
+      <c r="B91" t="n">
+        <v>0</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>4470</v>
+      </c>
+      <c r="B92" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>4475</v>
+      </c>
+      <c r="B93" t="n">
+        <v>0</v>
+      </c>
+      <c r="C93" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>4480</v>
+      </c>
+      <c r="B94" t="n">
+        <v>0</v>
+      </c>
+      <c r="C94" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>4485</v>
+      </c>
+      <c r="B95" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>4490</v>
+      </c>
+      <c r="B96" t="n">
+        <v>0</v>
+      </c>
+      <c r="C96" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>4495</v>
+      </c>
+      <c r="B97" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>4500</v>
+      </c>
+      <c r="B98" t="n">
+        <v>1</v>
+      </c>
+      <c r="C98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>4505</v>
+      </c>
+      <c r="B99" t="n">
+        <v>0</v>
+      </c>
+      <c r="C99" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="100"/>
     <row r="101"/>
     <row r="102"/>
@@ -7735,7 +8182,7 @@
         </is>
       </c>
       <c r="J6" s="45" t="n">
-        <v>4186.7</v>
+        <v>4162.3</v>
       </c>
       <c r="AB6">
         <f>IF(NOT(ISNUMBER('Gamma Data'!A6)),"",IF((ABS('Gamma Data'!B6)+ABS('Gamma Data'!C6))=0,"",IF(OR(ABS('Gamma Data'!A6-$J$6)&gt;$J$6*$J$26,ABS('Gamma Data'!A6-$J$6)&lt;$J$28),"",(ABS('Gamma Data'!B6)+ABS('Gamma Data'!C6))/MAX(ABS('Gamma Data'!A6-$J$6)/($J$6*0.005),1)+ROW()/1000000000)))</f>
@@ -17651,7 +18098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.42578125" bestFit="1" customWidth="1" style="61" min="1" max="1"/>
@@ -17880,6 +18327,52 @@
       </c>
       <c r="N5" s="32" t="n">
         <v>0.4087403598971722</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="71" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>G1MV6</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="n">
+        <v>4162.3</v>
+      </c>
+      <c r="D6" s="29" t="n">
+        <v>280</v>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>339</v>
+      </c>
+      <c r="F6" s="29" t="n">
+        <v>-59</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Negative GEX (วิ่ง)</t>
+        </is>
+      </c>
+      <c r="H6" s="29" t="n"/>
+      <c r="I6" s="29" t="n">
+        <v>4170</v>
+      </c>
+      <c r="J6" s="73" t="n">
+        <v>46298.64884631945</v>
+      </c>
+      <c r="K6" s="29" t="n">
+        <v>4190</v>
+      </c>
+      <c r="L6" s="29" t="n">
+        <v>4150</v>
+      </c>
+      <c r="M6" s="29" t="n">
+        <v>4190</v>
+      </c>
+      <c r="N6" s="32" t="n">
+        <v>0.170028818443804</v>
       </c>
     </row>
   </sheetData>
@@ -17893,7 +18386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y6"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18283,7 +18776,7 @@
         </is>
       </c>
       <c r="Q6" s="73" t="n">
-        <v>46298.43735601926</v>
+        <v>46298.43735601852</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -18293,7 +18786,7 @@
       <c r="S6" s="30" t="n">
         <v>4190.1</v>
       </c>
-      <c r="T6" s="74" t="n">
+      <c r="T6" s="75" t="n">
         <v>7</v>
       </c>
       <c r="U6" t="inlineStr">
@@ -18313,6 +18806,210 @@
       <c r="Y6" s="29" t="n">
         <v>4225</v>
       </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="71" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AB1 Week 5 - SEP 2026 (U26)</t>
+        </is>
+      </c>
+      <c r="C7" s="71" t="n">
+        <v>46294</v>
+      </c>
+      <c r="D7" s="30" t="n">
+        <v>4136.4</v>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>4200</v>
+      </c>
+      <c r="F7" s="29" t="n"/>
+      <c r="G7" s="29" t="n"/>
+      <c r="H7" s="30" t="n">
+        <v>4147.7</v>
+      </c>
+      <c r="I7" s="30" t="n">
+        <v>4185.4</v>
+      </c>
+      <c r="J7" s="30" t="n">
+        <v>4116.3</v>
+      </c>
+      <c r="K7" s="30" t="n">
+        <v>63.60000000000036</v>
+      </c>
+      <c r="L7" s="30" t="n">
+        <v>52.30000000000018</v>
+      </c>
+      <c r="M7" s="30" t="n">
+        <v>11.30000000000018</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" s="31" t="n">
+        <v>0.0167053476452953</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="Q7" s="73" t="n">
+        <v>46298.65528628538</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>OCT 26</t>
+        </is>
+      </c>
+      <c r="S7" s="30" t="n">
+        <v>4117.6</v>
+      </c>
+      <c r="T7" s="75" t="n">
+        <v>-151.4</v>
+      </c>
+      <c r="V7" s="32" t="n"/>
+      <c r="W7" s="29" t="n"/>
+      <c r="X7" s="29" t="n"/>
+      <c r="Y7" s="29" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="71" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>WD1 Week 5 - SEP 2026 (U26)</t>
+        </is>
+      </c>
+      <c r="C8" s="71" t="n">
+        <v>46295</v>
+      </c>
+      <c r="D8" s="30" t="n">
+        <v>4147.7</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>4235</v>
+      </c>
+      <c r="F8" s="29" t="n"/>
+      <c r="G8" s="29" t="n"/>
+      <c r="H8" s="30" t="n">
+        <v>4155.6</v>
+      </c>
+      <c r="I8" s="30" t="n">
+        <v>4217.4</v>
+      </c>
+      <c r="J8" s="30" t="n">
+        <v>4151.4</v>
+      </c>
+      <c r="K8" s="30" t="n">
+        <v>87.30000000000018</v>
+      </c>
+      <c r="L8" s="30" t="n">
+        <v>79.39999999999964</v>
+      </c>
+      <c r="M8" s="30" t="n">
+        <v>7.900000000000546</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" s="31" t="n">
+        <v>0.01591243339682234</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="Q8" s="73" t="n">
+        <v>46298.65528985655</v>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>OCT 26</t>
+        </is>
+      </c>
+      <c r="S8" s="30" t="n">
+        <v>4183.8</v>
+      </c>
+      <c r="T8" s="75" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="V8" s="32" t="n"/>
+      <c r="W8" s="29" t="n"/>
+      <c r="X8" s="29" t="n"/>
+      <c r="Y8" s="29" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="71" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>E21 Week 1 - OCT 2026 (V26)</t>
+        </is>
+      </c>
+      <c r="C9" s="71" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D9" s="30" t="n">
+        <v>4202.3</v>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>4250</v>
+      </c>
+      <c r="F9" s="29" t="n"/>
+      <c r="G9" s="29" t="n"/>
+      <c r="H9" s="30" t="n">
+        <v>4162.3</v>
+      </c>
+      <c r="I9" s="30" t="n">
+        <v>4259</v>
+      </c>
+      <c r="J9" s="30" t="n">
+        <v>4153.8</v>
+      </c>
+      <c r="K9" s="30" t="n">
+        <v>47.69999999999982</v>
+      </c>
+      <c r="L9" s="30" t="n">
+        <v>87.69999999999982</v>
+      </c>
+      <c r="M9" s="30" t="n">
+        <v>40</v>
+      </c>
+      <c r="N9" t="b">
+        <v>0</v>
+      </c>
+      <c r="O9" s="31" t="n">
+        <v>0.02503391000166571</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="Q9" s="73" t="n">
+        <v>46298.65529687911</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>DEC 26</t>
+        </is>
+      </c>
+      <c r="S9" s="30" t="n">
+        <v>4204.6</v>
+      </c>
+      <c r="T9" s="75" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="V9" s="32" t="n"/>
+      <c r="W9" s="29" t="n"/>
+      <c r="X9" s="29" t="n"/>
+      <c r="Y9" s="29" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>